<commit_message>
Fixed the write code file issue
</commit_message>
<xml_diff>
--- a/project_review.xlsx
+++ b/project_review.xlsx
@@ -725,12 +725,12 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>❌</t>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
@@ -777,7 +777,7 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -829,12 +829,12 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>❌</t>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
@@ -867,7 +867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -892,7 +892,7 @@
     <row r="4" ht="40" customHeight="1">
       <c r="A4" s="9" t="inlineStr">
         <is>
-          <t>Error:</t>
+          <t>Chart 1 - Review Checklist</t>
         </is>
       </c>
       <c r="B4" s="10" t="n"/>
@@ -901,7 +901,7 @@
     <row r="5" ht="40" customHeight="1">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>Incorrect CSS Link: The &lt;link&gt; tag references stylesssss.css, but the project file is named style.css.</t>
+          <t>Chart 2 - API Calls Summary</t>
         </is>
       </c>
       <c r="B5" s="10" t="n"/>
@@ -910,7 +910,7 @@
     <row r="6" ht="40" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>Accessibility: The &lt;img&gt; tag for the QR code has an empty alt attribute.</t>
+          <t>Chart 3 - Security Issues / Best Practices</t>
         </is>
       </c>
       <c r="B6" s="10" t="n"/>
@@ -919,7 +919,7 @@
     <row r="7" ht="40" customHeight="1">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>Fixed code:</t>
+          <t>Error Analysis:</t>
         </is>
       </c>
       <c r="B7" s="10" t="n"/>
@@ -928,7 +928,7 @@
     <row r="8" ht="40" customHeight="1">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>Chart 1 - Review Checklist</t>
+          <t>CSS Linkage: The code attempts to link to stylessss.css, but the provided file is style.css.</t>
         </is>
       </c>
       <c r="B8" s="10" t="n"/>
@@ -937,7 +937,7 @@
     <row r="9" ht="40" customHeight="1">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>Chart 2 - API Calls Summary</t>
+          <t>JS Linkage: The code attempts to link to app.js, but the provided file is script.js.</t>
         </is>
       </c>
       <c r="B9" s="10" t="n"/>
@@ -946,7 +946,7 @@
     <row r="10" ht="40" customHeight="1">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>Chart 3 - Security Issues / Best Practices</t>
+          <t>Fixed code:</t>
         </is>
       </c>
       <c r="B10" s="10" t="n"/>
@@ -1027,7 +1027,7 @@
       </c>
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -1037,9 +1037,9 @@
           <t>Comments &amp; docs</t>
         </is>
       </c>
-      <c r="B19" s="16" t="inlineStr">
-        <is>
-          <t>❌</t>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -1109,16 +1109,8 @@
           <t>None</t>
         </is>
       </c>
-      <c r="B26" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C26" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
+      <c r="B26" s="13" t="inlineStr"/>
+      <c r="C26" s="13" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="12" t="inlineStr">
@@ -1142,24 +1134,12 @@
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
         <is>
-          <t>Resource Integrity</t>
+          <t>Content Security Policy</t>
         </is>
       </c>
       <c r="B30" s="13" t="inlineStr">
         <is>
-          <t>Use Subresource Integrity (SRI) hashes for Google Font links if possible to ensure they aren't tampered with.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="15" t="inlineStr">
-        <is>
-          <t>Accessibility</t>
-        </is>
-      </c>
-      <c r="B31" s="15" t="inlineStr">
-        <is>
-          <t>Always provide descriptive alt text for images used as functional components.</t>
+          <t>Add a CSP meta tag to restrict script sources and API calls to trusted domains.</t>
         </is>
       </c>
     </row>
@@ -1188,7 +1168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1213,7 +1193,7 @@
     <row r="4" ht="40" customHeight="1">
       <c r="A4" s="9" t="inlineStr">
         <is>
-          <t>Error:</t>
+          <t>Chart 1 - Review Checklist</t>
         </is>
       </c>
       <c r="B4" s="10" t="n"/>
@@ -1222,7 +1202,7 @@
     <row r="5" ht="40" customHeight="1">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>Syntax Error: asynchronous is not a valid keyword. It should be async.</t>
+          <t>Chart 2 - API Calls Summary</t>
         </is>
       </c>
       <c r="B5" s="10" t="n"/>
@@ -1231,7 +1211,7 @@
     <row r="6" ht="40" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>Logic/Runtime Error: fetch is an asynchronous operation but was called without await.</t>
+          <t>Chart 3 - Security Issues / Best Practices</t>
         </is>
       </c>
       <c r="B6" s="10" t="n"/>
@@ -1240,7 +1220,7 @@
     <row r="7" ht="40" customHeight="1">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>Missing Error Handling: The API call was not wrapped in a try...catch block as per requirements.</t>
+          <t>Error Analysis:</t>
         </is>
       </c>
       <c r="B7" s="10" t="n"/>
@@ -1249,7 +1229,7 @@
     <row r="8" ht="40" customHeight="1">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>Encoding Issue: The input value is appended directly to the URL without encodeURIComponent, which will break if the user enters characters like &amp; or #.</t>
+          <t>Syntax Error: asynchronous is not a valid JavaScript keyword; it must be async.</t>
         </is>
       </c>
       <c r="B8" s="10" t="n"/>
@@ -1258,7 +1238,7 @@
     <row r="9" ht="40" customHeight="1">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>UI Feedback: The "Loading..." text is never hidden if the logic fails or completes unless manually set.</t>
+          <t>Logic Error (Async): The fetch function returns a promise. Simply accessing .url from a Promise object without await is incorrect.</t>
         </is>
       </c>
       <c r="B9" s="10" t="n"/>
@@ -1267,7 +1247,7 @@
     <row r="10" ht="40" customHeight="1">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>Fixed code:</t>
+          <t>Missing Error Handling: No try...catch block around the API call as requested.</t>
         </is>
       </c>
       <c r="B10" s="10" t="n"/>
@@ -1276,7 +1256,7 @@
     <row r="11" ht="40" customHeight="1">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>Chart 1 - Review Checklist</t>
+          <t>UI Feedback: The loader element is hidden immediately because the code is synchronous and doesn't wait for the network response to finalize.</t>
         </is>
       </c>
       <c r="B11" s="10" t="n"/>
@@ -1285,44 +1265,47 @@
     <row r="12" ht="40" customHeight="1">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>Chart 2 - API Calls Summary</t>
+          <t>Fixed code:</t>
         </is>
       </c>
       <c r="B12" s="10" t="n"/>
       <c r="C12" s="11" t="n"/>
     </row>
-    <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>Chart 3 - Security Issues / Best Practices</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="n"/>
-      <c r="C13" s="11" t="n"/>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>Review Checklist</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="inlineStr">
-        <is>
-          <t>Review Checklist</t>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Review Aspect</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Review Aspect</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Status</t>
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>Variable naming</t>
+        </is>
+      </c>
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="inlineStr">
-        <is>
-          <t>Variable naming</t>
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>Hardcoded values/secrets</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -1332,9 +1315,9 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="15" t="inlineStr">
-        <is>
-          <t>Hardcoded values/secrets</t>
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>Code repetition</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
@@ -1344,9 +1327,9 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="13" t="inlineStr">
-        <is>
-          <t>Code repetition</t>
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>Modularity</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
@@ -1356,178 +1339,165 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="15" t="inlineStr">
-        <is>
-          <t>Modularity</t>
-        </is>
-      </c>
-      <c r="B20" s="14" t="inlineStr">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>Complexity (high/med/low)</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>Comments &amp; docs</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>Exception handling present</t>
+        </is>
+      </c>
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
+          <t>Dependency/import correctness</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="13" t="inlineStr">
-        <is>
-          <t>Complexity (high/med/low)</t>
-        </is>
-      </c>
-      <c r="B21" s="13" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="15" t="inlineStr">
-        <is>
-          <t>Comments &amp; docs</t>
-        </is>
-      </c>
-      <c r="B22" s="16" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>Security concerns</t>
+        </is>
+      </c>
+      <c r="B24" s="16" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="13" t="inlineStr">
-        <is>
-          <t>Exception handling present</t>
-        </is>
-      </c>
-      <c r="B23" s="16" t="inlineStr">
-        <is>
-          <t>❌</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="15" t="inlineStr">
-        <is>
-          <t>Dependency/import correctness</t>
-        </is>
-      </c>
-      <c r="B24" s="14" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="13" t="inlineStr">
-        <is>
-          <t>Security concerns</t>
-        </is>
-      </c>
-      <c r="B25" s="16" t="inlineStr">
-        <is>
-          <t>❌</t>
+    <row r="26">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>API Calls Summary</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="12" t="inlineStr">
-        <is>
-          <t>API Calls Summary</t>
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>API Endpoint</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Request (sample)</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Response (sample)</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>API Endpoint</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>Request (sample)</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>Response (sample)</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="13" t="inlineStr">
+      <c r="A28" s="13" t="inlineStr">
         <is>
           <t>https://api.qrserver.com/v1/create-qr-code/</t>
         </is>
       </c>
-      <c r="B29" s="13" t="inlineStr">
-        <is>
-          <t>GET ?size=150x150&amp;data=hello</t>
-        </is>
-      </c>
-      <c r="C29" s="13" t="inlineStr">
-        <is>
-          <t>(Image/PNG Data)</t>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>?size=150x150&amp;data=example</t>
+        </is>
+      </c>
+      <c r="C28" s="13" t="inlineStr">
+        <is>
+          <t>(Image Blob/File)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>Security / Best Practices</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="12" t="inlineStr">
-        <is>
-          <t>Security / Best Practices</t>
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Recommendation</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>Recommendation</t>
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>Input Validation</t>
+        </is>
+      </c>
+      <c r="B32" s="13" t="inlineStr">
+        <is>
+          <t>Use encodeURIComponent when passing user input into a URL to prevent URL breakage or potential injection.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="13" t="inlineStr">
-        <is>
-          <t>Input Sanitization</t>
-        </is>
-      </c>
-      <c r="B33" s="13" t="inlineStr">
-        <is>
-          <t>Use encodeURIComponent() when building URLs from user input to prevent URL injection/malformation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="15" t="inlineStr">
-        <is>
-          <t>Error Swallowing</t>
-        </is>
-      </c>
-      <c r="B34" s="15" t="inlineStr">
-        <is>
-          <t>Always catch promise rejections to prevent unhandled rejection errors in the console.</t>
+      <c r="A33" s="15" t="inlineStr">
+        <is>
+          <t>Error Handling</t>
+        </is>
+      </c>
+      <c r="B33" s="15" t="inlineStr">
+        <is>
+          <t>Implement try...catch blocks for network requests to handle downtime or invalid responses.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="14">
     <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A30:B30"/>
     <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A15:B15"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="A8:C8"/>
     <mergeCell ref="A6:C6"/>
     <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A14:B14"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="A7:C7"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A26:C26"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1539,7 +1509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1564,7 +1534,7 @@
     <row r="4" ht="40" customHeight="1">
       <c r="A4" s="9" t="inlineStr">
         <is>
-          <t>Error:</t>
+          <t>Chart 1 - Review Checklist</t>
         </is>
       </c>
       <c r="B4" s="10" t="n"/>
@@ -1573,7 +1543,7 @@
     <row r="5" ht="40" customHeight="1">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>Requirement Violation: The user requested the body background color to be green.</t>
+          <t>Chart 2 - API Calls Summary</t>
         </is>
       </c>
       <c r="B5" s="10" t="n"/>
@@ -1582,7 +1552,7 @@
     <row r="6" ht="40" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>Invalid CSS Value: #imgBox { width: 100; } is missing units (e.g., px or %). Browsers will ignore this property.</t>
+          <t>Chart 3 - Security Issues / Best Practices</t>
         </is>
       </c>
       <c r="B6" s="10" t="n"/>
@@ -1591,7 +1561,7 @@
     <row r="7" ht="40" customHeight="1">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>UI Improvement: The invalid-input class is applied to a &lt;p&gt; tag but has properties like border and background-color that might clash with the layout if not managed.</t>
+          <t>Error Analysis:</t>
         </is>
       </c>
       <c r="B7" s="10" t="n"/>
@@ -1600,7 +1570,7 @@
     <row r="8" ht="40" customHeight="1">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>Fixed code:</t>
+          <t>Requirement: User requested the body color to be green.</t>
         </is>
       </c>
       <c r="B8" s="10" t="n"/>
@@ -1609,7 +1579,7 @@
     <row r="9" ht="40" customHeight="1">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>Chart 1 - Review Checklist</t>
+          <t>Invalid Unit: #imgBox { width: 100; } is invalid CSS. It needs a unit like 100% or 100px.</t>
         </is>
       </c>
       <c r="B9" s="10" t="n"/>
@@ -1618,44 +1588,47 @@
     <row r="10" ht="40" customHeight="1">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>Chart 2 - API Calls Summary</t>
+          <t>Fixed code:</t>
         </is>
       </c>
       <c r="B10" s="10" t="n"/>
       <c r="C10" s="11" t="n"/>
     </row>
-    <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>Chart 3 - Security Issues / Best Practices</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="n"/>
-      <c r="C11" s="11" t="n"/>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>Review Checklist</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
-        <is>
-          <t>Review Checklist</t>
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Review Aspect</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Review Aspect</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Status</t>
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>Variable naming</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="inlineStr">
-        <is>
-          <t>Variable naming</t>
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>Hardcoded values/secrets</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
@@ -1665,9 +1638,9 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="15" t="inlineStr">
-        <is>
-          <t>Hardcoded values/secrets</t>
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>Code repetition</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
@@ -1677,9 +1650,9 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="inlineStr">
-        <is>
-          <t>Code repetition</t>
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>Modularity</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -1689,57 +1662,57 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="15" t="inlineStr">
-        <is>
-          <t>Modularity</t>
-        </is>
-      </c>
-      <c r="B18" s="14" t="inlineStr">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>Complexity (high/med/low)</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>Comments &amp; docs</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="13" t="inlineStr">
-        <is>
-          <t>Complexity (high/med/low)</t>
-        </is>
-      </c>
-      <c r="B19" s="13" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-    </row>
     <row r="20">
-      <c r="A20" s="15" t="inlineStr">
-        <is>
-          <t>Comments &amp; docs</t>
-        </is>
-      </c>
-      <c r="B20" s="16" t="inlineStr">
-        <is>
-          <t>❌</t>
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>Exception handling present</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="inlineStr">
-        <is>
-          <t>Exception handling present</t>
-        </is>
-      </c>
-      <c r="B21" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>Dependency/import correctness</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="15" t="inlineStr">
-        <is>
-          <t>Dependency/import correctness</t>
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>Security concerns</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr">
@@ -1748,117 +1721,84 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="13" t="inlineStr">
-        <is>
-          <t>Security concerns</t>
-        </is>
-      </c>
-      <c r="B23" s="14" t="inlineStr">
-        <is>
-          <t>✅</t>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>API Calls Summary</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="12" t="inlineStr">
-        <is>
-          <t>API Calls Summary</t>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>API Endpoint</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Request (sample)</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Response (sample)</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>API Endpoint</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Request (sample)</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>Response (sample)</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="13" t="inlineStr">
+      <c r="A26" s="13" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="B27" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C27" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="B26" s="13" t="inlineStr"/>
+      <c r="C26" s="13" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>Security / Best Practices</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="12" t="inlineStr">
-        <is>
-          <t>Security / Best Practices</t>
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Recommendation</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>Recommendation</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="13" t="inlineStr">
-        <is>
-          <t>CSS Unit Validation</t>
-        </is>
-      </c>
-      <c r="B31" s="13" t="inlineStr">
-        <is>
-          <t>Always specify units (px, %, em) for non-zero numerical values to ensure cross-browser compatibility.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="15" t="inlineStr">
-        <is>
-          <t>User Experience</t>
-        </is>
-      </c>
-      <c r="B32" s="15" t="inlineStr">
-        <is>
-          <t>Ensure text colors inside the invalid-input state have sufficient contrast against the background.</t>
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>CSS is standard.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="12">
     <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A25:C25"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A29:B29"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="A8:C8"/>
     <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A28:B28"/>
     <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A13:B13"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="A7:C7"/>
     <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="A12:B12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1870,7 +1810,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A252"/>
+  <dimension ref="A1:A262"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -1886,7 +1826,7 @@
     <row r="3">
       <c r="A3" s="18" t="inlineStr">
         <is>
-          <t>### FILE PATH: C:/Users/ashay/Downloads/Quiz/QR-Code-Generator\index.html</t>
+          <t>## Project Analysis: QR Code Generator</t>
         </is>
       </c>
     </row>
@@ -1896,21 +1836,17 @@
     <row r="5">
       <c r="A5" s="18" t="inlineStr">
         <is>
-          <t>**Error:**</t>
+          <t>The project consists of a simple web application to generate QR codes using an external API. There are several critical syntax and linkage errors that prevent the code from running, along with logic issues in handling asynchronous operations.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>1.  **Incorrect CSS Link:** The `&lt;link&gt;` tag references `stylesssss.css`, but the project file is named `style.css`.</t>
-        </is>
-      </c>
+      <c r="A6" s="18" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="18" t="inlineStr">
         <is>
-          <t>2.  **Accessibility:** The `&lt;img&gt;` tag for the QR code has an empty `alt` attribute.</t>
+          <t>---</t>
         </is>
       </c>
     </row>
@@ -1920,196 +1856,180 @@
     <row r="9">
       <c r="A9" s="18" t="inlineStr">
         <is>
-          <t>**Fixed code:**</t>
+          <t>### FILE PATH: C:/Users/ashay/Downloads/Quiz/QR-Code-Generator\index.html</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>```html</t>
-        </is>
-      </c>
+      <c r="A10" s="18" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="18" t="inlineStr">
         <is>
-          <t>&lt;!DOCTYPE html&gt;</t>
+          <t>**Chart 1 - Review Checklist**</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="18" t="inlineStr">
         <is>
-          <t>&lt;html lang="en"&gt;</t>
+          <t>| Review Aspect | Status |</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="18" t="inlineStr">
         <is>
-          <t>&lt;head&gt;</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    &lt;meta charset="UTF-8"&gt;</t>
+          <t>| Variable naming | ✅ |</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    &lt;meta name="viewport" content="width=device-width, initial-scale=1.0"&gt;</t>
+          <t>| Hardcoded values/secrets | ✅ |</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    &lt;title&gt;QR Code Generator&lt;/title&gt;</t>
+          <t>| Code repetition | ✅ |</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    </t>
+          <t>| Modularity | ✅ |</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    &lt;link rel="preconnect" href="https://fonts.googleapis.com"&gt;</t>
+          <t>| Complexity (high/med/low) | Low |</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    &lt;link rel="preconnect" href="https://fonts.gstatic.com" crossorigin&gt;</t>
+          <t>| Comments &amp; docs | ✅ |</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    &lt;link href="https://fonts.googleapis.com/css2?family=Poppins:ital,wght@0,100;0,200;0,300;0,400;0,500;0,600;0,700;0,800;0,900;1,100;1,200;1,300;1,400;1,500;1,600;1,700;1,800;1,900&amp;display=swap" rel="stylesheet"&gt;</t>
+          <t>| Exception handling present | N/A |</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    &lt;!-- Fixed: Corrected filename from stylesssss.css to style.css --&gt;</t>
+          <t>| Dependency/import correctness | ❌ |</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    &lt;link rel="stylesheet" href="style.css"&gt;</t>
+          <t>| Security concerns | ✅ |</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="18" t="inlineStr">
-        <is>
-          <t>&lt;/head&gt;</t>
-        </is>
-      </c>
+      <c r="A23" s="18" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="18" t="inlineStr">
         <is>
-          <t>&lt;body&gt;</t>
+          <t>**Chart 2 - API Calls Summary**</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    &lt;div class="container"&gt;</t>
+          <t>| API Endpoint | Request (sample) | Response (sample) |</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">        &lt;p&gt;Enter Text or URL here&lt;/p&gt;</t>
+          <t>|---|---|---|</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">        &lt;input type="text" placeholder="eg : www.google.com" id="Qr-text"&gt;</t>
+          <t>| None | | |</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        &lt;div id="imgBox"&gt;</t>
-        </is>
-      </c>
+      <c r="A28" s="18" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">            &lt;img src="" alt="QR Code Output" id="Qr-Image"&gt;</t>
+          <t>**Chart 3 - Security Issues / Best Practices**</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">        &lt;/div&gt;</t>
+          <t>| Category | Recommendation |</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">        &lt;button&gt;Generate QR Code&lt;/button&gt;</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    &lt;/div&gt;</t>
+          <t>| Content Security Policy | Add a CSP meta tag to restrict script sources and API calls to trusted domains. |</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    &lt;script src="script.js"&gt;&lt;/script&gt;</t>
-        </is>
-      </c>
+      <c r="A33" s="18" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="18" t="inlineStr">
         <is>
-          <t>&lt;/body&gt;</t>
+          <t>**Error Analysis:**</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="18" t="inlineStr">
         <is>
-          <t>&lt;/html&gt;</t>
+          <t>1.  **CSS Linkage:** The code attempts to link to `stylessss.css`, but the provided file is `style.css`.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="18" t="inlineStr">
         <is>
-          <t>```</t>
+          <t>2.  **JS Linkage:** The code attempts to link to `app.js`, but the provided file is `script.js`.</t>
         </is>
       </c>
     </row>
@@ -2119,794 +2039,806 @@
     <row r="38">
       <c r="A38" s="18" t="inlineStr">
         <is>
-          <t>**Chart 1 - Review Checklist**</t>
+          <t>**Fixed code:**</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="18" t="inlineStr">
         <is>
-          <t>| Review Aspect | Status |</t>
+          <t>```html</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="18" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t>&lt;!DOCTYPE html&gt;</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="18" t="inlineStr">
         <is>
-          <t>| Variable naming | ✅ |</t>
+          <t>&lt;html lang="en"&gt;</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="18" t="inlineStr">
         <is>
-          <t>| Hardcoded values/secrets | ✅ |</t>
+          <t>&lt;head&gt;</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="18" t="inlineStr">
         <is>
-          <t>| Code repetition | ✅ |</t>
+          <t xml:space="preserve">    &lt;meta charset="UTF-8"&gt;</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="18" t="inlineStr">
         <is>
-          <t>| Modularity | ✅ |</t>
+          <t xml:space="preserve">    &lt;meta name="viewport" content="width=device-width, initial-scale=1.0"&gt;</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="18" t="inlineStr">
         <is>
-          <t>| Complexity (high/med/low) | low |</t>
+          <t xml:space="preserve">    &lt;title&gt;QR Code Generator&lt;/title&gt;</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="18" t="inlineStr">
         <is>
-          <t>| Comments &amp; docs | ❌ |</t>
+          <t xml:space="preserve">    </t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="18" t="inlineStr">
         <is>
-          <t>| Exception handling present | N/A |</t>
+          <t xml:space="preserve">    &lt;link rel="preconnect" href="https://fonts.googleapis.com"&gt;</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="18" t="inlineStr">
         <is>
-          <t>| Dependency/import correctness | ❌ |</t>
+          <t xml:space="preserve">    &lt;link rel="preconnect" href="https://fonts.gstatic.com" crossorigin&gt;</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="18" t="inlineStr">
         <is>
-          <t>| Security concerns | ✅ |</t>
+          <t xml:space="preserve">    &lt;link href="https://fonts.googleapis.com/css2?family=Poppins:ital,wght@0,100;0,200;0,300;0,400;0,500;0,600;0,700;0,800;0,900;1,100;1,200;1,300;1,400;1,500;1,600;1,700;1,800;1,900&amp;display=swap" rel="stylesheet"&gt;</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="18" t="inlineStr"/>
+      <c r="A50" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    &lt;!-- Fixed link name from stylessss.css to style.css --&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="18" t="inlineStr">
         <is>
-          <t>**Chart 2 - API Calls Summary**</t>
+          <t xml:space="preserve">    &lt;link rel="stylesheet" href="style.css"&gt;</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="18" t="inlineStr">
         <is>
-          <t>| API Endpoint | Request (sample) | Response (sample) |</t>
+          <t>&lt;/head&gt;</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="18" t="inlineStr">
         <is>
-          <t>|---|---|---|</t>
+          <t>&lt;body&gt;</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="18" t="inlineStr">
         <is>
-          <t>| None | N/A | N/A |</t>
+          <t xml:space="preserve">    &lt;div class="container"&gt;</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="18" t="inlineStr"/>
+      <c r="A55" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        &lt;p&gt;Enter Text or URL here&lt;/p&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="18" t="inlineStr">
         <is>
-          <t>**Chart 3 - Security Issues / Best Practices**</t>
+          <t xml:space="preserve">        &lt;input type="text" placeholder="eg : www.google.com" id="Qr-text"&gt;</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="18" t="inlineStr">
         <is>
-          <t>| Category | Recommendation |</t>
+          <t xml:space="preserve">        &lt;div id="imgBox"&gt;</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="18" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t xml:space="preserve">            &lt;img src="" alt="" id="Qr-Image"&gt;</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="18" t="inlineStr">
         <is>
-          <t>| Resource Integrity | Use Subresource Integrity (SRI) hashes for Google Font links if possible to ensure they aren't tampered with. |</t>
+          <t xml:space="preserve">        &lt;/div&gt;</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="18" t="inlineStr">
         <is>
-          <t>| Accessibility | Always provide descriptive `alt` text for images used as functional components. |</t>
+          <t xml:space="preserve">        &lt;button&gt;Generate QR Code&lt;/button&gt;</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="18" t="inlineStr"/>
+      <c r="A61" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    &lt;/div&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="18" t="inlineStr">
         <is>
-          <t>---</t>
+          <t xml:space="preserve">    &lt;!-- Fixed link name from app.js to script.js --&gt;</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="18" t="inlineStr"/>
+      <c r="A63" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    &lt;script src="script.js"&gt;&lt;/script&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="18" t="inlineStr">
         <is>
-          <t>### FILE PATH: C:/Users/ashay/Downloads/Quiz/QR-Code-Generator\script.js</t>
+          <t>&lt;/body&gt;</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="18" t="inlineStr"/>
+      <c r="A65" s="18" t="inlineStr">
+        <is>
+          <t>&lt;/html&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="18" t="inlineStr">
         <is>
-          <t>**Error:**</t>
+          <t>```</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="18" t="inlineStr">
-        <is>
-          <t>1.  **Syntax Error:** `asynchronous` is not a valid keyword. It should be `async`.</t>
-        </is>
-      </c>
+      <c r="A67" s="18" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="18" t="inlineStr">
         <is>
-          <t>2.  **Logic/Runtime Error:** `fetch` is an asynchronous operation but was called without `await`.</t>
+          <t>---</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="18" t="inlineStr">
-        <is>
-          <t>3.  **Missing Error Handling:** The API call was not wrapped in a `try...catch` block as per requirements.</t>
-        </is>
-      </c>
+      <c r="A69" s="18" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="18" t="inlineStr">
         <is>
-          <t>4.  **Encoding Issue:** The input value is appended directly to the URL without `encodeURIComponent`, which will break if the user enters characters like `&amp;` or `#`.</t>
+          <t>### FILE PATH: C:/Users/ashay/Downloads/Quiz/QR-Code-Generator\script.js</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="18" t="inlineStr">
-        <is>
-          <t>5.  **UI Feedback:** The "Loading..." text is never hidden if the logic fails or completes unless manually set.</t>
-        </is>
-      </c>
+      <c r="A71" s="18" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" s="18" t="inlineStr"/>
+      <c r="A72" s="18" t="inlineStr">
+        <is>
+          <t>**Chart 1 - Review Checklist**</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="18" t="inlineStr">
         <is>
-          <t>**Fixed code:**</t>
+          <t>| Review Aspect | Status |</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="18" t="inlineStr">
         <is>
-          <t>```javascript</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="18" t="inlineStr">
         <is>
-          <t>const btn = document.querySelector('button');</t>
+          <t>| Variable naming | ✅ |</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="18" t="inlineStr">
         <is>
-          <t>const imgbox = document.getElementById('imgBox');</t>
+          <t>| Hardcoded values/secrets | ✅ |</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="18" t="inlineStr">
         <is>
-          <t>const qrImage = document.getElementById('Qr-Image');</t>
+          <t>| Code repetition | ✅ |</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="18" t="inlineStr">
         <is>
-          <t>const input = document.getElementById('Qr-text');</t>
+          <t>| Modularity | ✅ |</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="18" t="inlineStr">
         <is>
-          <t>const loadelement = document.createElement('p');</t>
+          <t>| Complexity (high/med/low) | Low |</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="18" t="inlineStr">
         <is>
-          <t>imgbox.append(loadelement);</t>
+          <t>| Comments &amp; docs | ❌ |</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="18" t="inlineStr"/>
+      <c r="A81" s="18" t="inlineStr">
+        <is>
+          <t>| Exception handling present | ❌ |</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="18" t="inlineStr">
         <is>
-          <t>const getQR = async () =&gt; {</t>
+          <t>| Dependency/import correctness | ✅ |</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    loadelement.hidden = false;</t>
+          <t>| Security concerns | ❌ |</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    </t>
-        </is>
-      </c>
+      <c r="A84" s="18" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    if (input.value.trim().length &gt; 0) {</t>
+          <t>**Chart 2 - API Calls Summary**</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">        qrImage.src = '';</t>
+          <t>| API Endpoint | Request (sample) | Response (sample) |</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">        loadelement.classList.remove('invalid-input');</t>
+          <t>|---|---|---|</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">        loadelement.innerHTML = 'Loading ...';</t>
+          <t>| `https://api.qrserver.com/v1/create-qr-code/` | `?size=150x150&amp;data=example` | (Image Blob/File) |</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        </t>
-        </is>
-      </c>
+      <c r="A89" s="18" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">        try {</t>
+          <t>**Chart 3 - Security Issues / Best Practices**</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">            // URL encode the input to handle special characters correctly</t>
+          <t>| Category | Recommendation |</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">            const apiUrl = `https://api.qrserver.com/v1/create-qr-code/?size=150x150&amp;data=${encodeURIComponent(input.value)}`;</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">            </t>
+          <t>| Input Validation | Use `encodeURIComponent` when passing user input into a URL to prevent URL breakage or potential injection. |</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">            const response = await fetch(apiUrl);</t>
+          <t>| Error Handling | Implement `try...catch` blocks for network requests to handle downtime or invalid responses. |</t>
         </is>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">            </t>
-        </is>
-      </c>
+      <c r="A95" s="18" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">            if (!response.ok) {</t>
+          <t>**Error Analysis:**</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">                throw new Error('Network response was not ok');</t>
+          <t>1.  **Syntax Error:** `asynchronous` is not a valid JavaScript keyword; it must be `async`.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">            }</t>
+          <t>2.  **Logic Error (Async):** The `fetch` function returns a promise. Simply accessing `.url` from a Promise object without `await` is incorrect.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">            </t>
+          <t>3.  **Missing Error Handling:** No `try...catch` block around the API call as requested.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">            // For this specific API, the URL itself is the source for the image</t>
+          <t>4.  **UI Feedback:** The loader element is hidden immediately because the code is synchronous and doesn't wait for the network response to finalize.</t>
         </is>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">            qrImage.src = response.url;</t>
-        </is>
-      </c>
+      <c r="A101" s="18" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">            loadelement.hidden = true;</t>
+          <t>**Fixed code:**</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">        } catch (error) {</t>
+          <t>```javascript</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">            console.error('Error fetching QR code:', error);</t>
+          <t>const btn = document.getElementsByTagName('button')[0];</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">            loadelement.innerHTML = 'Error fetching QR Code. Try again.';</t>
+          <t>const imgbox = document.getElementById('imgBox');</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">            loadelement.classList.add('invalid-input');</t>
+          <t>const qrImage = document.getElementById('Qr-Image');</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">        }</t>
+          <t>const input = document.getElementById('Qr-text');</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    } else {</t>
+          <t>const loadelement = document.createElement('p');</t>
         </is>
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        qrImage.src = '';</t>
-        </is>
-      </c>
+      <c r="A109" s="18" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">        loadelement.classList.add('invalid-input');</t>
+          <t>imgbox.append(loadelement);</t>
         </is>
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        loadelement.innerHTML = 'Invalid Input !';</t>
-        </is>
-      </c>
+      <c r="A111" s="18" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">        loadelement.hidden = false;</t>
+          <t>/**</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    }</t>
+          <t xml:space="preserve"> * Fetches QR code from API and updates the UI.</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="18" t="inlineStr">
         <is>
-          <t>}</t>
+          <t xml:space="preserve"> * Corrected 'asynchronous' to 'async' and added try-catch.</t>
         </is>
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="18" t="inlineStr"/>
+      <c r="A115" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> */</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="18" t="inlineStr">
         <is>
-          <t>btn.addEventListener('click', getQR);</t>
+          <t>const getQR = async () =&gt; {</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="18" t="inlineStr">
         <is>
-          <t>```</t>
+          <t xml:space="preserve">    loadelement.hidden = false;</t>
         </is>
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="18" t="inlineStr"/>
+      <c r="A118" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    </t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="18" t="inlineStr">
         <is>
-          <t>**Chart 1 - Review Checklist**</t>
+          <t xml:space="preserve">    if (input.value.trim().length &gt; 0) {</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="18" t="inlineStr">
         <is>
-          <t>| Review Aspect | Status |</t>
+          <t xml:space="preserve">        qrImage.src = '';</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="18" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t xml:space="preserve">        loadelement.classList.remove('invalid-input');</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="18" t="inlineStr">
         <is>
-          <t>| Variable naming | ✅ |</t>
+          <t xml:space="preserve">        loadelement.innerHTML = 'Loading ...';</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="18" t="inlineStr">
         <is>
-          <t>| Hardcoded values/secrets | ✅ |</t>
+          <t xml:space="preserve">        </t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="18" t="inlineStr">
         <is>
-          <t>| Code repetition | ✅ |</t>
+          <t xml:space="preserve">        try {</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="18" t="inlineStr">
         <is>
-          <t>| Modularity | ✅ |</t>
+          <t xml:space="preserve">            // Encode the input to handle special characters correctly</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="18" t="inlineStr">
         <is>
-          <t>| Complexity (high/med/low) | low |</t>
+          <t xml:space="preserve">            const apiUrl = `https://api.qrserver.com/v1/create-qr-code/?size=150x150&amp;data=${encodeURIComponent(input.value)}`;</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="18" t="inlineStr">
         <is>
-          <t>| Comments &amp; docs | ❌ |</t>
+          <t xml:space="preserve">            </t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="18" t="inlineStr">
         <is>
-          <t>| Exception handling present | ❌ |</t>
+          <t xml:space="preserve">            const response = await fetch(apiUrl);</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="18" t="inlineStr">
         <is>
-          <t>| Dependency/import correctness | ✅ |</t>
+          <t xml:space="preserve">            </t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="18" t="inlineStr">
         <is>
-          <t>| Security concerns | ❌ |</t>
+          <t xml:space="preserve">            if (!response.ok) {</t>
         </is>
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="18" t="inlineStr"/>
+      <c r="A131" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                throw new Error('Network response was not ok');</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="18" t="inlineStr">
         <is>
-          <t>**Chart 2 - API Calls Summary**</t>
+          <t xml:space="preserve">            }</t>
         </is>
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="18" t="inlineStr">
-        <is>
-          <t>| API Endpoint | Request (sample) | Response (sample) |</t>
-        </is>
-      </c>
+      <c r="A133" s="18" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="18" t="inlineStr">
         <is>
-          <t>|---|---|---|</t>
+          <t xml:space="preserve">            // Setting image src to the response URL</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="18" t="inlineStr">
         <is>
-          <t>| `https://api.qrserver.com/v1/create-qr-code/` | GET `?size=150x150&amp;data=hello` | (Image/PNG Data) |</t>
+          <t xml:space="preserve">            qrImage.src = response.url;</t>
         </is>
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="18" t="inlineStr"/>
+      <c r="A136" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            </t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="18" t="inlineStr">
         <is>
-          <t>**Chart 3 - Security Issues / Best Practices**</t>
+          <t xml:space="preserve">            // Wait for image to load before hiding the loader for better UX</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="18" t="inlineStr">
         <is>
-          <t>| Category | Recommendation |</t>
+          <t xml:space="preserve">            qrImage.onload = () =&gt; {</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="18" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t xml:space="preserve">                loadelement.hidden = true;</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="18" t="inlineStr">
         <is>
-          <t>| Input Sanitization | Use `encodeURIComponent()` when building URLs from user input to prevent URL injection/malformation. |</t>
+          <t xml:space="preserve">            };</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="18" t="inlineStr">
         <is>
-          <t>| Error Swallowing | Always catch promise rejections to prevent unhandled rejection errors in the console. |</t>
+          <t xml:space="preserve">            </t>
         </is>
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="18" t="inlineStr"/>
+      <c r="A142" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        } catch (error) {</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="18" t="inlineStr">
         <is>
-          <t>---</t>
+          <t xml:space="preserve">            console.error("Fetch error:", error);</t>
         </is>
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="18" t="inlineStr"/>
+      <c r="A144" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            loadelement.classList.add('invalid-input');</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="18" t="inlineStr">
         <is>
-          <t>### FILE PATH: C:/Users/ashay/Downloads/Quiz/QR-Code-Generator\style.css</t>
+          <t xml:space="preserve">            loadelement.innerHTML = 'Error fetching QR Code!';</t>
         </is>
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="18" t="inlineStr"/>
+      <c r="A146" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            loadelement.hidden = false;</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="18" t="inlineStr">
         <is>
-          <t>**Error:**</t>
+          <t xml:space="preserve">        }</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="18" t="inlineStr">
         <is>
-          <t>1.  **Requirement Violation:** The user requested the body background color to be green.</t>
+          <t xml:space="preserve">    } else {</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="18" t="inlineStr">
         <is>
-          <t>2.  **Invalid CSS Value:** `#imgBox { width: 100; }` is missing units (e.g., `px` or `%`). Browsers will ignore this property.</t>
+          <t xml:space="preserve">        qrImage.src = '';</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="18" t="inlineStr">
         <is>
-          <t>3.  **UI Improvement:** The `invalid-input` class is applied to a `&lt;p&gt;` tag but has properties like `border` and `background-color` that might clash with the layout if not managed.</t>
+          <t xml:space="preserve">        loadelement.classList.add('invalid-input');</t>
         </is>
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="18" t="inlineStr"/>
+      <c r="A151" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        loadelement.innerHTML = 'Invalid Input !';</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="18" t="inlineStr">
         <is>
-          <t>**Fixed code:**</t>
+          <t xml:space="preserve">        loadelement.hidden = false;</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="18" t="inlineStr">
         <is>
-          <t>```css</t>
+          <t xml:space="preserve">    }</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="18" t="inlineStr">
         <is>
-          <t>*{</t>
+          <t>}</t>
         </is>
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    margin: 0;</t>
-        </is>
-      </c>
+      <c r="A155" s="18" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    padding: 0;</t>
+          <t>btn.addEventListener('click', getQR);</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    font-family :'Poppins', sans-serif;</t>
+          <t>```</t>
         </is>
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    box-sizing: border-box;</t>
-        </is>
-      </c>
+      <c r="A158" s="18" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" s="18" t="inlineStr">
         <is>
-          <t>}</t>
+          <t>---</t>
         </is>
       </c>
     </row>
@@ -2916,600 +2848,662 @@
     <row r="161">
       <c r="A161" s="18" t="inlineStr">
         <is>
-          <t>body{</t>
+          <t>### FILE PATH: C:/Users/ashay/Downloads/Quiz/QR-Code-Generator\style.css</t>
         </is>
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    /* Requirement: Make body color green */</t>
-        </is>
-      </c>
+      <c r="A162" s="18" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    background-color: #28a745;</t>
+          <t>**Chart 1 - Review Checklist**</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="18" t="inlineStr">
         <is>
-          <t>}</t>
+          <t>| Review Aspect | Status |</t>
         </is>
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="18" t="inlineStr"/>
+      <c r="A165" s="18" t="inlineStr">
+        <is>
+          <t>|---|---|</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="18" t="inlineStr">
         <is>
-          <t>.container{</t>
+          <t>| Variable naming | ✅ |</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    width : 400px;</t>
+          <t>| Hardcoded values/secrets | ✅ |</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    background-color: white;</t>
+          <t>| Code repetition | ✅ |</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    border-radius: 10px;  </t>
+          <t>| Modularity | ✅ |</t>
         </is>
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="18" t="inlineStr"/>
+      <c r="A170" s="18" t="inlineStr">
+        <is>
+          <t>| Complexity (high/med/low) | Low |</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    /* Centering the div */</t>
+          <t>| Comments &amp; docs | ✅ |</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    padding: 25px 35px;</t>
+          <t>| Exception handling present | N/A |</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    position:absolute;</t>
+          <t>| Dependency/import correctness | ✅ |</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    top : 50%;</t>
+          <t>| Security concerns | ✅ |</t>
         </is>
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    left: 50%;</t>
-        </is>
-      </c>
+      <c r="A175" s="18" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    transform: translate(-50%, -50%);  </t>
+          <t>**Chart 2 - API Calls Summary**</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="18" t="inlineStr">
         <is>
-          <t>}</t>
+          <t>| API Endpoint | Request (sample) | Response (sample) |</t>
         </is>
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="18" t="inlineStr"/>
+      <c r="A178" s="18" t="inlineStr">
+        <is>
+          <t>|---|---|---|</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="18" t="inlineStr">
         <is>
-          <t>.container p{</t>
+          <t>| None | | |</t>
         </is>
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    font-weight: 600;</t>
-        </is>
-      </c>
+      <c r="A180" s="18" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    font-size: 15px;</t>
+          <t>**Chart 3 - Security Issues / Best Practices**</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    margin-bottom: 8px;</t>
+          <t>| Category | Recommendation |</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="18" t="inlineStr">
         <is>
-          <t>}</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="18" t="inlineStr"/>
+      <c r="A184" s="18" t="inlineStr">
+        <is>
+          <t>| None | CSS is standard. |</t>
+        </is>
+      </c>
     </row>
     <row r="185">
-      <c r="A185" s="18" t="inlineStr">
-        <is>
-          <t>.container input{</t>
-        </is>
-      </c>
+      <c r="A185" s="18" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    width: 100%;</t>
+          <t>**Error Analysis:**</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    height: 50px;</t>
+          <t>1.  **Requirement:** User requested the body color to be green.</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    border: 1px solid #494eea;</t>
+          <t>2.  **Invalid Unit:** `#imgBox { width: 100; }` is invalid CSS. It needs a unit like `100%` or `100px`.</t>
         </is>
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    outline: 0;</t>
-        </is>
-      </c>
+      <c r="A189" s="18" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    padding: 10px;</t>
+          <t>**Fixed code:**</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    margin: 10px 0 20px;</t>
+          <t>```css</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    border-radius: 5px;</t>
+          <t>*{</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="18" t="inlineStr">
         <is>
-          <t>}</t>
+          <t xml:space="preserve">    margin: 0;</t>
         </is>
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="18" t="inlineStr"/>
+      <c r="A194" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    padding: 0;</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="18" t="inlineStr">
         <is>
-          <t>.container button{</t>
+          <t xml:space="preserve">    font-family :'Poppins', sans-serif;</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    width: 100%;</t>
+          <t xml:space="preserve">    box-sizing: border-box;</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    height: 50px;</t>
+          <t>}</t>
         </is>
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    border : 0;</t>
-        </is>
-      </c>
+      <c r="A198" s="18" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    background-color: #494eea;</t>
+          <t>body{</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    color: white;</t>
+          <t xml:space="preserve">    /* Requirement: Body color set to green */</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    outline: 0;</t>
+          <t xml:space="preserve">    background-color: #2ecc71;</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    border-radius: 5px;</t>
+          <t>}</t>
         </is>
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    margin:20px 0;</t>
-        </is>
-      </c>
+      <c r="A203" s="18" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    font-weight: 500;</t>
+          <t>.container{</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    cursor: pointer;</t>
+          <t xml:space="preserve">    width : 400px;</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="18" t="inlineStr">
         <is>
-          <t>}</t>
+          <t xml:space="preserve">    background-color: white;</t>
         </is>
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="18" t="inlineStr"/>
+      <c r="A207" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    border-radius: 10px;  </t>
+        </is>
+      </c>
     </row>
     <row r="208">
-      <c r="A208" s="18" t="inlineStr">
-        <is>
-          <t>#imgBox{</t>
-        </is>
-      </c>
+      <c r="A208" s="18" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    /* Fixed: Added % unit */</t>
+          <t xml:space="preserve">    /* Centering the div */</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    width: 100%;</t>
+          <t xml:space="preserve">    padding: 25px 35px;</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    display: flex;</t>
+          <t xml:space="preserve">    position:absolute;</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    justify-content: center;</t>
+          <t xml:space="preserve">    top : 50%;</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    min-height: 10px;</t>
+          <t xml:space="preserve">    left: 50%;</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="18" t="inlineStr">
         <is>
+          <t xml:space="preserve">    transform: translate(-50%, -50%);  </t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="18" t="inlineStr">
+        <is>
           <t>}</t>
         </is>
       </c>
     </row>
-    <row r="215">
-      <c r="A215" s="18" t="inlineStr"/>
-    </row>
     <row r="216">
-      <c r="A216" s="18" t="inlineStr">
-        <is>
-          <t>#Qr-Image {</t>
-        </is>
-      </c>
+      <c r="A216" s="18" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    max-width: 150px;</t>
+          <t>.container p{</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="18" t="inlineStr">
         <is>
-          <t>}</t>
+          <t xml:space="preserve">    font-weight: 600;</t>
         </is>
       </c>
     </row>
     <row r="219">
-      <c r="A219" s="18" t="inlineStr"/>
+      <c r="A219" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    font-size: 15px;</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="18" t="inlineStr">
         <is>
-          <t>.invalid-input{</t>
+          <t xml:space="preserve">    margin-bottom: 8px;</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    border: 2px solid red;</t>
+          <t>}</t>
         </is>
       </c>
     </row>
     <row r="222">
-      <c r="A222" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    background-color: rgb(232, 132, 132);</t>
-        </is>
-      </c>
+      <c r="A222" s="18" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    color: white;</t>
+          <t>.container input{</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    border-radius: 3px;</t>
+          <t xml:space="preserve">    width: 100%;</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    padding: 5px;</t>
+          <t xml:space="preserve">    height: 50px;</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    text-align: center;</t>
+          <t xml:space="preserve">    border: 1px solid #494eea;</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="18" t="inlineStr">
         <is>
-          <t>}</t>
+          <t xml:space="preserve">    outline: 0;</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="18" t="inlineStr">
         <is>
-          <t>```</t>
+          <t xml:space="preserve">    padding: 10px;</t>
         </is>
       </c>
     </row>
     <row r="229">
-      <c r="A229" s="18" t="inlineStr"/>
+      <c r="A229" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    margin: 10px 0 20px;</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="18" t="inlineStr">
         <is>
-          <t>**Chart 1 - Review Checklist**</t>
+          <t xml:space="preserve">    border-radius: 5px;</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="18" t="inlineStr">
         <is>
-          <t>| Review Aspect | Status |</t>
+          <t>}</t>
         </is>
       </c>
     </row>
     <row r="232">
-      <c r="A232" s="18" t="inlineStr">
-        <is>
-          <t>|---|---|</t>
-        </is>
-      </c>
+      <c r="A232" s="18" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" s="18" t="inlineStr">
         <is>
-          <t>| Variable naming | ✅ |</t>
+          <t>.container button{</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="18" t="inlineStr">
         <is>
-          <t>| Hardcoded values/secrets | ✅ |</t>
+          <t xml:space="preserve">    width: 100%;</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="18" t="inlineStr">
         <is>
-          <t>| Code repetition | ✅ |</t>
+          <t xml:space="preserve">    height: 50px;</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="18" t="inlineStr">
         <is>
-          <t>| Modularity | ✅ |</t>
+          <t xml:space="preserve">    border : 0;</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="18" t="inlineStr">
         <is>
-          <t>| Complexity (high/med/low) | low |</t>
+          <t xml:space="preserve">    background-color: #494eea;</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="18" t="inlineStr">
         <is>
-          <t>| Comments &amp; docs | ❌ |</t>
+          <t xml:space="preserve">    color: white;</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="18" t="inlineStr">
         <is>
-          <t>| Exception handling present | N/A |</t>
+          <t xml:space="preserve">    outline: 0;</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="18" t="inlineStr">
         <is>
-          <t>| Dependency/import correctness | ✅ |</t>
+          <t xml:space="preserve">    border-radius: 5px;</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="18" t="inlineStr">
         <is>
-          <t>| Security concerns | ✅ |</t>
+          <t xml:space="preserve">    margin:20px 0;</t>
         </is>
       </c>
     </row>
     <row r="242">
-      <c r="A242" s="18" t="inlineStr"/>
+      <c r="A242" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    font-weight: 500;</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="18" t="inlineStr">
         <is>
-          <t>**Chart 2 - API Calls Summary**</t>
+          <t xml:space="preserve">    cursor: pointer;</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="18" t="inlineStr">
         <is>
-          <t>| API Endpoint | Request (sample) | Response (sample) |</t>
+          <t>}</t>
         </is>
       </c>
     </row>
     <row r="245">
-      <c r="A245" s="18" t="inlineStr">
-        <is>
-          <t>|---|---|---|</t>
-        </is>
-      </c>
+      <c r="A245" s="18" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" s="18" t="inlineStr">
         <is>
-          <t>| None | N/A | N/A |</t>
+          <t>#imgBox{</t>
         </is>
       </c>
     </row>
     <row r="247">
-      <c r="A247" s="18" t="inlineStr"/>
+      <c r="A247" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    /* Fixed: Added unit to width */</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" s="18" t="inlineStr">
         <is>
-          <t>**Chart 3 - Security Issues / Best Practices**</t>
+          <t xml:space="preserve">    width: 100%;</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="18" t="inlineStr">
         <is>
-          <t>| Category | Recommendation |</t>
+          <t xml:space="preserve">    display: flex;</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="18" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t xml:space="preserve">    justify-content: center;</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="18" t="inlineStr">
         <is>
-          <t>| CSS Unit Validation | Always specify units (px, %, em) for non-zero numerical values to ensure cross-browser compatibility. |</t>
+          <t>}</t>
         </is>
       </c>
     </row>
     <row r="252">
-      <c r="A252" s="18" t="inlineStr">
-        <is>
-          <t>| User Experience | Ensure text colors inside the `invalid-input` state have sufficient contrast against the background. |</t>
+      <c r="A252" s="18" t="inlineStr"/>
+    </row>
+    <row r="253">
+      <c r="A253" s="18" t="inlineStr">
+        <is>
+          <t>.invalid-input{</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    border: 2px solid red;</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    background-color: rgb(232, 132, 132);</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    color: white;</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    border-radius: 3px;</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    padding: 5px;</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    text-align: center;</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    width: 100%;</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="18" t="inlineStr">
+        <is>
+          <t>}</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="18" t="inlineStr">
+        <is>
+          <t>```</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tested and working fine
</commit_message>
<xml_diff>
--- a/project_review.xlsx
+++ b/project_review.xlsx
@@ -119,7 +119,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C8E6C9"/>
+        <fgColor rgb="00FFCDD2"/>
       </patternFill>
     </fill>
     <fill>
@@ -129,7 +129,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFCDD2"/>
+        <fgColor rgb="00C8E6C9"/>
       </patternFill>
     </fill>
     <fill>
@@ -183,10 +183,10 @@
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -657,45 +657,45 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>❌</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="J3" s="5" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -707,49 +707,49 @@
           <t>script.js</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>❌</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>❌</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
         </is>
       </c>
     </row>
@@ -759,47 +759,47 @@
           <t>style.css</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I5" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -819,7 +819,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -830,7 +830,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>📄  C:/Users/ashay/Downloads/test-code-debugger/QR-Code-Generator/index.html</t>
+          <t>📄  C:/Users/ashay/Downloads/test-code-debugger/QR-Code-Generator\index.html</t>
         </is>
       </c>
     </row>
@@ -868,7 +868,7 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>❌</t>
         </is>
       </c>
     </row>
@@ -878,7 +878,7 @@
           <t>Hardcoded values/secrets</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -890,7 +890,7 @@
           <t>Code repetition</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -902,7 +902,7 @@
           <t>Modularity</t>
         </is>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -926,7 +926,7 @@
           <t>Comments &amp; docs</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
@@ -940,7 +940,7 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>❌</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
           <t>Dependency/import correctness</t>
         </is>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="13" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -962,7 +962,7 @@
           <t>Security concerns</t>
         </is>
       </c>
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B15" s="13" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -1028,7 +1028,31 @@
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>Add a label for the input element to improve screen reader support.</t>
+          <t>Replace &lt;p&gt; with a &lt;label&gt; associated with the input for screen reader support.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>Use a transparent 1x1px data URI for src instead of an empty string to prevent the browser from attempting to load the page itself as an image.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>Best Practices</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>Use consistent naming conventions (e.g., camelCase or kebab-case) for IDs and add a unique ID to the button.</t>
         </is>
       </c>
     </row>
@@ -1050,7 +1074,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1061,7 +1085,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>📄  C:/Users/ashay/Downloads/test-code-debugger/QR-Code-Generator/script.js</t>
+          <t>📄  C:/Users/ashay/Downloads/test-code-debugger/QR-Code-Generator\script.js</t>
         </is>
       </c>
     </row>
@@ -1097,7 +1121,7 @@
           <t>Variable naming</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -1111,7 +1135,7 @@
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>❌</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1145,7 @@
           <t>Code repetition</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -1135,7 +1159,7 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>❌</t>
         </is>
       </c>
     </row>
@@ -1157,7 +1181,7 @@
           <t>Comments &amp; docs</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
@@ -1169,7 +1193,7 @@
           <t>Exception handling present</t>
         </is>
       </c>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
@@ -1181,7 +1205,7 @@
           <t>Dependency/import correctness</t>
         </is>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="13" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -1195,7 +1219,7 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>❌</t>
         </is>
       </c>
     </row>
@@ -1231,12 +1255,12 @@
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>GET /v1/create-qr-code/?size=150x150&amp;data=example</t>
+          <t>GET /?size=150x150&amp;data=Hello</t>
         </is>
       </c>
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t>Image file (PNG/JPG)</t>
+          <t>Image File (MIME: image/png)</t>
         </is>
       </c>
     </row>
@@ -1262,24 +1286,48 @@
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
         <is>
-          <t>Error Handling</t>
+          <t>Input Validation</t>
         </is>
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>Wrap the fetch call in a try...catch block to handle network errors and check response.ok.</t>
+          <t>Use encodeURIComponent() on input.value to ensure special characters (like &amp;, ?, #) don't break the API query string.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
         <is>
-          <t>Hardcoded Values</t>
+          <t>Exception Handling</t>
         </is>
       </c>
       <c r="B24" s="12" t="inlineStr">
         <is>
-          <t>Move the base API URL to a constant variable.</t>
+          <t>Wrap fetch calls in try...catch blocks to handle network timeouts or DNS failures gracefully.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>UX Improvement</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>Use input.value.trim() to prevent generating QR codes for empty whitespace.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>Logic Error</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>Verify response.ok before attempting to use the response, as fetch does not reject on 404 or 500 errors.</t>
         </is>
       </c>
     </row>
@@ -1301,7 +1349,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1312,7 +1360,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>📄  C:/Users/ashay/Downloads/test-code-debugger/QR-Code-Generator/style.css</t>
+          <t>📄  C:/Users/ashay/Downloads/test-code-debugger/QR-Code-Generator\style.css</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1396,7 @@
           <t>Variable naming</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -1362,7 +1410,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>❌</t>
         </is>
       </c>
     </row>
@@ -1372,7 +1420,7 @@
           <t>Code repetition</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -1384,7 +1432,7 @@
           <t>Modularity</t>
         </is>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -1410,7 +1458,7 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>❌</t>
         </is>
       </c>
     </row>
@@ -1420,7 +1468,7 @@
           <t>Exception handling present</t>
         </is>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="13" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -1432,7 +1480,7 @@
           <t>Dependency/import correctness</t>
         </is>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="13" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -1444,7 +1492,7 @@
           <t>Security concerns</t>
         </is>
       </c>
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B15" s="13" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -1505,12 +1553,36 @@
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
         <is>
-          <t>CSS Validation</t>
+          <t>Accessibility</t>
         </is>
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>Always provide units (px, %, em) for non-zero numeric values in CSS.</t>
+          <t>Use focus-visible or maintain outlines for keyboard navigation accessibility.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>Maintainability</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>Use CSS variables for repeated colors like #494eea.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>Compatibility</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>Always provide a generic fallback (e.g., sans-serif) for custom fonts.</t>
         </is>
       </c>
     </row>
@@ -1532,7 +1604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A244"/>
+  <dimension ref="A1:A258"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -1548,14 +1620,14 @@
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
-          <t>### FILE: C:/Users/ashay/Downloads/test-code-debugger/QR-Code-Generator/index.html</t>
+          <t>### FILE: C:/Users/ashay/Downloads/test-code-debugger/QR-Code-Generator\index.html</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
         <is>
-          <t>### Error: No errors found</t>
+          <t>### Error: Empty image source attribute causes redundant server requests, missing button identifier makes script targeting fragile, and lack of input labels reduces accessibility.</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1651,7 @@
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
         <is>
-          <t>| Variable naming | ✅ |</t>
+          <t>| Variable naming | ❌ |</t>
         </is>
       </c>
     </row>
@@ -1621,7 +1693,7 @@
     <row r="14">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>| Exception handling present | ✅ |</t>
+          <t>| Exception handling present | ❌ |</t>
         </is>
       </c>
     </row>
@@ -1683,619 +1755,611 @@
     <row r="24">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>| Accessibility | Add a label for the input element to improve screen reader support. |</t>
+          <t>| Accessibility | Replace `&lt;p&gt;` with a `&lt;label&gt;` associated with the input for screen reader support. |</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="15" t="inlineStr"/>
+      <c r="A25" s="15" t="inlineStr">
+        <is>
+          <t>| Performance | Use a transparent 1x1px data URI for `src` instead of an empty string to prevent the browser from attempting to load the page itself as an image. |</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>Fixed code:</t>
+          <t>| Best Practices | Use consistent naming conventions (e.g., camelCase or kebab-case) for IDs and add a unique ID to the button. |</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="15" t="inlineStr">
-        <is>
-          <t>```html</t>
-        </is>
-      </c>
+      <c r="A27" s="15" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>&lt;!DOCTYPE html&gt;</t>
+          <t>Fixed code:</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="15" t="inlineStr">
         <is>
-          <t>&lt;html lang="en"&gt;</t>
+          <t>```html</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="15" t="inlineStr">
         <is>
-          <t>&lt;head&gt;</t>
+          <t>&lt;!DOCTYPE html&gt;</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    &lt;meta charset="UTF-8"&gt;</t>
+          <t>&lt;html lang="en"&gt;</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    &lt;meta name="viewport" content="width=device-width, initial-scale=1.0"&gt;</t>
+          <t>&lt;head&gt;</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    &lt;title&gt;QR Code Generator&lt;/title&gt;</t>
+          <t xml:space="preserve">    &lt;meta charset="UTF-8"&gt;</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    </t>
+          <t xml:space="preserve">    &lt;meta name="viewport" content="width=device-width, initial-scale=1.0"&gt;</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    &lt;link rel="preconnect" href="https://fonts.googleapis.com"&gt;</t>
+          <t xml:space="preserve">    &lt;title&gt;QR Code Generator&lt;/title&gt;</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    &lt;link rel="preconnect" href="https://fonts.gstatic.com" crossorigin&gt;</t>
+          <t xml:space="preserve">    </t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    &lt;link href="https://fonts.googleapis.com/css2?family=Poppins:ital,wght@0,100;0,200;0,300;0,400;0,500;0,600;0,700;0,800;0,900;1,100;1,200;1,300;1,400;1,500;1,600;1,700;1,800;1,900&amp;display=swap" rel="stylesheet"&gt;</t>
+          <t xml:space="preserve">    &lt;!-- Preconnect to Google Fonts for performance --&gt;</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    &lt;link rel="stylesheet" href="style.css"&gt;</t>
+          <t xml:space="preserve">    &lt;link rel="preconnect" href="https://fonts.googleapis.com"&gt;</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="15" t="inlineStr">
         <is>
-          <t>&lt;/head&gt;</t>
+          <t xml:space="preserve">    &lt;link rel="preconnect" href="https://fonts.gstatic.com" crossorigin&gt;</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="15" t="inlineStr">
         <is>
-          <t>&lt;body&gt;</t>
+          <t xml:space="preserve">    &lt;!-- Poppins Font Import --&gt;</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    &lt;div class="container"&gt;</t>
+          <t xml:space="preserve">    &lt;link href="https://fonts.googleapis.com/css2?family=Poppins:ital,wght@0,100;0,200;0,300;0,400;0,500;0,600;0,700;0,800;0,900;1,100;1,200;1,300;1,400;1,500;1,600;1,700;1,800;1,900&amp;display=swap" rel="stylesheet"&gt;</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">        &lt;p&gt;Enter Text or URL here&lt;/p&gt;</t>
+          <t xml:space="preserve">    &lt;!-- Link to external stylesheet --&gt;</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">        &lt;label for="Qr-text" style="display:none;"&gt;QR Content&lt;/label&gt;</t>
+          <t xml:space="preserve">    &lt;link rel="stylesheet" href="style.css"&gt;</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">        &lt;input type="text" placeholder="eg : www.google.com" id="Qr-text"&gt;</t>
+          <t>&lt;/head&gt;</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">        &lt;div id="imgBox"&gt;</t>
+          <t>&lt;body&gt;</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">            &lt;img src="" alt="QR Code" id="Qr-Image"&gt;</t>
+          <t xml:space="preserve">    &lt;div class="container"&gt;</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">        &lt;/div&gt;</t>
+          <t xml:space="preserve">        &lt;!-- Improved accessibility with label tag --&gt;</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">        &lt;button type="button" id="generate-btn"&gt;Generate QR Code&lt;/button&gt;</t>
+          <t xml:space="preserve">        &lt;label for="qr-text"&gt;Enter Text or URL here&lt;/label&gt;</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    &lt;/div&gt;</t>
+          <t xml:space="preserve">        &lt;input type="text" placeholder="eg: www.google.com" id="qr-text" autocomplete="off"&gt;</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    &lt;script src="script.js"&gt;&lt;/script&gt;</t>
+          <t xml:space="preserve">        </t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="15" t="inlineStr">
         <is>
-          <t>&lt;/body&gt;</t>
+          <t xml:space="preserve">        &lt;div id="imgBox"&gt;</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="15" t="inlineStr">
         <is>
-          <t>&lt;/html&gt;</t>
+          <t xml:space="preserve">            &lt;!-- Used data URI to prevent broken image icon/404 on load --&gt;</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="15" t="inlineStr">
         <is>
-          <t>```</t>
+          <t xml:space="preserve">            &lt;img src="data:image/gif;base64,R0lGODlhAQABAIAAAAAAAP///yH5BAEAAAAALAAAAAABAAEAAAIBRAA7" alt="Generated QR Code" id="qr-image"&gt;</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="15" t="inlineStr"/>
+      <c r="A54" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        &lt;/div&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="15" t="inlineStr">
         <is>
-          <t>### FILE: C:/Users/ashay/Downloads/test-code-debugger/QR-Code-Generator/script.js</t>
+          <t xml:space="preserve">        </t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="15" t="inlineStr">
         <is>
-          <t>### Error: Missing try-catch block for the network request; lack of error handling for failed API responses or network timeouts.</t>
+          <t xml:space="preserve">        &lt;!-- Added ID for precise script selection --&gt;</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="15" t="inlineStr"/>
+      <c r="A57" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        &lt;button type="button" id="generate-btn"&gt;Generate QR Code&lt;/button&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="15" t="inlineStr">
         <is>
-          <t>| Review Aspect | Status |</t>
+          <t xml:space="preserve">    &lt;/div&gt;</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="15" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t xml:space="preserve">    </t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="15" t="inlineStr">
         <is>
-          <t>| Variable naming | ✅ |</t>
+          <t xml:space="preserve">    &lt;!-- Script included at the end of body for performance --&gt;</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="15" t="inlineStr">
         <is>
-          <t>| Hardcoded values/secrets | ❌ |</t>
+          <t xml:space="preserve">    &lt;script src="script.js"&gt;&lt;/script&gt;</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="15" t="inlineStr">
         <is>
-          <t>| Code repetition | ✅ |</t>
+          <t>&lt;/body&gt;</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="15" t="inlineStr">
         <is>
-          <t>| Modularity | ✅ |</t>
+          <t>&lt;/html&gt;</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="15" t="inlineStr">
         <is>
-          <t>| Complexity (high/med/low) | low |</t>
+          <t>```</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="15" t="inlineStr">
-        <is>
-          <t>| Comments &amp; docs | ❌ |</t>
-        </is>
-      </c>
+      <c r="A65" s="15" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="15" t="inlineStr">
         <is>
-          <t>| Exception handling present | ❌ |</t>
+          <t>### FILE: C:/Users/ashay/Downloads/test-code-debugger/QR-Code-Generator\script.js</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="15" t="inlineStr">
         <is>
-          <t>| Dependency/import correctness | ✅ |</t>
+          <t>### Error: Missing exception handling (try-catch) for asynchronous fetch operation; missing URL encoding for user input; no verification of response status; lack of input trimming.</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="15" t="inlineStr">
-        <is>
-          <t>| Security concerns | ✅ |</t>
-        </is>
-      </c>
+      <c r="A68" s="15" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" s="15" t="inlineStr"/>
+      <c r="A69" s="15" t="inlineStr">
+        <is>
+          <t>| Review Aspect | Status |</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="15" t="inlineStr">
         <is>
-          <t>| API Endpoint | Request (sample) | Response (sample) |</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="15" t="inlineStr">
         <is>
-          <t>|---|---|---|</t>
+          <t>| Variable naming | ✅ |</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="15" t="inlineStr">
         <is>
-          <t>| `https://api.qrserver.com/v1/create-qr-code/` | `GET /v1/create-qr-code/?size=150x150&amp;data=example` | Image file (PNG/JPG) |</t>
+          <t>| Hardcoded values/secrets | ✅ |</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="15" t="inlineStr"/>
+      <c r="A73" s="15" t="inlineStr">
+        <is>
+          <t>| Code repetition | ✅ |</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="15" t="inlineStr">
         <is>
-          <t>| Category | Recommendation |</t>
+          <t>| Modularity | ❌ |</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="15" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t>| Complexity (high/med/low) | low |</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="15" t="inlineStr">
         <is>
-          <t>| Error Handling | Wrap the `fetch` call in a `try...catch` block to handle network errors and check `response.ok`. |</t>
+          <t>| Comments &amp; docs | ❌ |</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="15" t="inlineStr">
         <is>
-          <t>| Hardcoded Values | Move the base API URL to a constant variable. |</t>
+          <t>| Exception handling present | ❌ |</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="15" t="inlineStr"/>
+      <c r="A78" s="15" t="inlineStr">
+        <is>
+          <t>| Dependency/import correctness | ✅ |</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="15" t="inlineStr">
         <is>
-          <t>Fixed code:</t>
+          <t>| Security concerns | ❌ |</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="15" t="inlineStr">
-        <is>
-          <t>```js</t>
-        </is>
-      </c>
+      <c r="A80" s="15" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="15" t="inlineStr">
         <is>
-          <t>const btn = document.querySelector('button');</t>
+          <t>| API Endpoint | Request (sample) | Response (sample) |</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="15" t="inlineStr">
         <is>
-          <t>const imgbox = document.getElementById('imgBox');</t>
+          <t>|---|---|---|</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="15" t="inlineStr">
         <is>
-          <t>const qrImage = document.getElementById('Qr-Image');</t>
+          <t>| `https://api.qrserver.com/v1/create-qr-code/` | `GET /?size=150x150&amp;data=Hello` | Image File (MIME: image/png) |</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="15" t="inlineStr">
-        <is>
-          <t>const input = document.getElementById('Qr-text');</t>
-        </is>
-      </c>
+      <c r="A84" s="15" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="15" t="inlineStr">
         <is>
-          <t>const loadelement = document.createElement('p');</t>
+          <t>| Category | Recommendation |</t>
         </is>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="15" t="inlineStr"/>
+      <c r="A86" s="15" t="inlineStr">
+        <is>
+          <t>|---|---|</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="15" t="inlineStr">
         <is>
-          <t>imgbox.append(loadelement);</t>
+          <t>| Input Validation | Use `encodeURIComponent()` on `input.value` to ensure special characters (like &amp;, ?, #) don't break the API query string. |</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="15" t="inlineStr">
         <is>
-          <t>loadelement.hidden = true;</t>
+          <t>| Exception Handling | Wrap `fetch` calls in `try...catch` blocks to handle network timeouts or DNS failures gracefully. |</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="15" t="inlineStr"/>
+      <c r="A89" s="15" t="inlineStr">
+        <is>
+          <t>| UX Improvement | Use `input.value.trim()` to prevent generating QR codes for empty whitespace. |</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="15" t="inlineStr">
         <is>
-          <t>const getQR = async () =&gt; {</t>
+          <t>| Logic Error | Verify `response.ok` before attempting to use the response, as `fetch` does not reject on 404 or 500 errors. |</t>
         </is>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    const inputValue = input.value.trim();</t>
-        </is>
-      </c>
+      <c r="A91" s="15" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    </t>
+          <t>Fixed code:</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    if (inputValue.length &gt; 0) {</t>
+          <t>```js</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">        loadelement.hidden = false;</t>
+          <t>const btn = document.getElementsByTagName('button')[0];</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">        qrImage.src = '';</t>
+          <t>const imgbox = document.getElementById('imgBox');</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">        qrImage.style.display = 'none';</t>
+          <t>const qrImage = document.getElementById('Qr-Image');</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">        loadelement.classList.remove('invalid-input');</t>
+          <t>const input = document.getElementById('Qr-text');</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">        loadelement.innerHTML = 'Loading ...';</t>
+          <t>const loadelement = document.createElement('p');</t>
         </is>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        </t>
-        </is>
-      </c>
+      <c r="A99" s="15" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">        const apiUrl = `https://api.qrserver.com/v1/create-qr-code/?size=150x150&amp;data=${encodeURIComponent(inputValue)}`;</t>
+          <t>imgbox.append(loadelement);</t>
         </is>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        </t>
-        </is>
-      </c>
+      <c r="A101" s="15" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">        try {</t>
+          <t>/**</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">            const response = await fetch(apiUrl);</t>
+          <t xml:space="preserve"> * Fetches and displays a QR code based on user input.</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">            </t>
+          <t xml:space="preserve"> */</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">            if (!response.ok) {</t>
+          <t>const getQR = async () =&gt; {</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">                throw new Error('Network response was not ok');</t>
+          <t xml:space="preserve">    const trimmedValue = input.value.trim();</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">            }</t>
+          <t xml:space="preserve">    loadelement.hidden = false;</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">            </t>
+          <t xml:space="preserve">    loadelement.classList.remove('invalid-input');</t>
         </is>
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">            // For this specific API, the URL itself is the source</t>
-        </is>
-      </c>
+      <c r="A109" s="15" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">            qrImage.src = response.url;</t>
+          <t xml:space="preserve">    if (trimmedValue.length &gt; 0) {</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">            </t>
+          <t xml:space="preserve">        try {</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">            // Wait for image to actually load before hiding loader</t>
+          <t xml:space="preserve">            qrImage.src = '';</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">            qrImage.onload = () =&gt; {</t>
+          <t xml:space="preserve">            loadelement.innerHTML = 'Loading ...';</t>
         </is>
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">                loadelement.hidden = true;</t>
-        </is>
-      </c>
+      <c r="A114" s="15" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">                qrImage.style.display = 'block';</t>
+          <t xml:space="preserve">            // Use encodeURIComponent to handle special characters in input</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">            };</t>
+          <t xml:space="preserve">            const apiUrl = `https://api.qrserver.com/v1/create-qr-code/?size=150x150&amp;data=${encodeURIComponent(trimmedValue)}`;</t>
         </is>
       </c>
     </row>
@@ -2309,139 +2373,139 @@
     <row r="118">
       <c r="A118" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">            qrImage.onerror = () =&gt; {</t>
+          <t xml:space="preserve">            const response = await fetch(apiUrl);</t>
         </is>
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">                throw new Error('Image failed to load');</t>
-        </is>
-      </c>
+      <c r="A119" s="15" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">            };</t>
+          <t xml:space="preserve">            if (!response.ok) {</t>
         </is>
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="15" t="inlineStr"/>
+      <c r="A121" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                throw new Error(`HTTP error! status: ${response.status}`);</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">        } catch (error) {</t>
+          <t xml:space="preserve">            }</t>
         </is>
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">            console.error('Fetch error:', error);</t>
-        </is>
-      </c>
+      <c r="A123" s="15" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">            loadelement.classList.add('invalid-input');</t>
+          <t xml:space="preserve">            // Setting src directly from response.url</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">            loadelement.innerHTML = 'Error fetching QR Code!';</t>
+          <t xml:space="preserve">            qrImage.src = response.url;</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">            loadelement.hidden = false;</t>
+          <t xml:space="preserve">            loadelement.hidden = true;</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">        }</t>
+          <t xml:space="preserve">        } catch (error) {</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    } else {</t>
+          <t xml:space="preserve">            console.error('Error generating QR code:', error);</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">        qrImage.src = '';</t>
+          <t xml:space="preserve">            qrImage.src = '';</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">        qrImage.style.display = 'none';</t>
+          <t xml:space="preserve">            loadelement.classList.add('invalid-input');</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">        loadelement.hidden = false;</t>
+          <t xml:space="preserve">            loadelement.innerHTML = 'Service Unavailable. Try again later.';</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">        loadelement.classList.add('invalid-input');</t>
+          <t xml:space="preserve">        }</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">        loadelement.innerHTML = 'Invalid Input !';</t>
+          <t xml:space="preserve">    } else {</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    }</t>
+          <t xml:space="preserve">        qrImage.src = '';</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="15" t="inlineStr">
         <is>
-          <t>};</t>
+          <t xml:space="preserve">        loadelement.classList.add('invalid-input');</t>
         </is>
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="15" t="inlineStr"/>
+      <c r="A136" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        loadelement.innerHTML = 'Invalid Input !';</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="15" t="inlineStr">
         <is>
-          <t>btn.addEventListener('click', getQR);</t>
+          <t xml:space="preserve">    }</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="15" t="inlineStr">
         <is>
-          <t>```</t>
+          <t>};</t>
         </is>
       </c>
     </row>
@@ -2451,14 +2515,14 @@
     <row r="140">
       <c r="A140" s="15" t="inlineStr">
         <is>
-          <t>### FILE: C:/Users/ashay/Downloads/test-code-debugger/QR-Code-Generator/style.css</t>
+          <t>btn.addEventListener('click', getQR);</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="15" t="inlineStr">
         <is>
-          <t>### Error: Syntax error in #imgBox; width value "100" is missing a unit (e.g., px, %).</t>
+          <t>```</t>
         </is>
       </c>
     </row>
@@ -2468,440 +2532,436 @@
     <row r="143">
       <c r="A143" s="15" t="inlineStr">
         <is>
-          <t>| Review Aspect | Status |</t>
+          <t>### FILE: C:/Users/ashay/Downloads/test-code-debugger/QR-Code-Generator\style.css</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="15" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t>### Error: Syntax error in `#imgBox` width unit and missing fallback font families for better compatibility.</t>
         </is>
       </c>
     </row>
     <row r="145">
-      <c r="A145" s="15" t="inlineStr">
-        <is>
-          <t>| Variable naming | ✅ |</t>
-        </is>
-      </c>
+      <c r="A145" s="15" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="15" t="inlineStr">
         <is>
-          <t>| Hardcoded values/secrets | ✅ |</t>
+          <t>| Review Aspect | Status |</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="15" t="inlineStr">
         <is>
-          <t>| Code repetition | ✅ |</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="15" t="inlineStr">
         <is>
-          <t>| Modularity | ✅ |</t>
+          <t>| Variable naming | ✅ |</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="15" t="inlineStr">
         <is>
-          <t>| Complexity (high/med/low) | low |</t>
+          <t>| Hardcoded values/secrets | ❌ |</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="15" t="inlineStr">
         <is>
-          <t>| Comments &amp; docs | ✅ |</t>
+          <t>| Code repetition | ✅ |</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="15" t="inlineStr">
         <is>
-          <t>| Exception handling present | ✅ |</t>
+          <t>| Modularity | ✅ |</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="15" t="inlineStr">
         <is>
-          <t>| Dependency/import correctness | ✅ |</t>
+          <t>| Complexity (high/med/low) | low |</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="15" t="inlineStr">
         <is>
-          <t>| Security concerns | ✅ |</t>
+          <t>| Comments &amp; docs | ❌ |</t>
         </is>
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="15" t="inlineStr"/>
+      <c r="A154" s="15" t="inlineStr">
+        <is>
+          <t>| Exception handling present | ✅ |</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="15" t="inlineStr">
         <is>
-          <t>| API Endpoint | Request (sample) | Response (sample) |</t>
+          <t>| Dependency/import correctness | ✅ |</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="15" t="inlineStr">
         <is>
-          <t>|---|---|---|</t>
+          <t>| Security concerns | ✅ |</t>
         </is>
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="15" t="inlineStr">
-        <is>
-          <t>| None | | |</t>
-        </is>
-      </c>
+      <c r="A157" s="15" t="inlineStr"/>
     </row>
     <row r="158">
-      <c r="A158" s="15" t="inlineStr"/>
+      <c r="A158" s="15" t="inlineStr">
+        <is>
+          <t>| API Endpoint | Request (sample) | Response (sample) |</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="15" t="inlineStr">
         <is>
-          <t>| Category | Recommendation |</t>
+          <t>|---|---|---|</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="15" t="inlineStr">
         <is>
-          <t>|---|---|</t>
+          <t>| None | | |</t>
         </is>
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="15" t="inlineStr">
-        <is>
-          <t>| CSS Validation | Always provide units (px, %, em) for non-zero numeric values in CSS. |</t>
-        </is>
-      </c>
+      <c r="A161" s="15" t="inlineStr"/>
     </row>
     <row r="162">
-      <c r="A162" s="15" t="inlineStr"/>
+      <c r="A162" s="15" t="inlineStr">
+        <is>
+          <t>| Category | Recommendation |</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="15" t="inlineStr">
         <is>
-          <t>Fixed code:</t>
+          <t>|---|---|</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="15" t="inlineStr">
         <is>
-          <t>```css</t>
+          <t>| Accessibility | Use focus-visible or maintain outlines for keyboard navigation accessibility. |</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="15" t="inlineStr">
         <is>
-          <t>*{</t>
+          <t>| Maintainability | Use CSS variables for repeated colors like `#494eea`. |</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    margin: 0;</t>
+          <t>| Compatibility | Always provide a generic fallback (e.g., `sans-serif`) for custom fonts. |</t>
         </is>
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    padding: 0;</t>
-        </is>
-      </c>
+      <c r="A167" s="15" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    font-family :'Poppins', sans-serif;</t>
+          <t>Fixed code:</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    box-sizing: border-box;</t>
+          <t>```css</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="15" t="inlineStr">
         <is>
-          <t>}</t>
+          <t>*{</t>
         </is>
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="15" t="inlineStr"/>
+      <c r="A171" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    margin: 0;</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="15" t="inlineStr">
         <is>
-          <t>body{</t>
+          <t xml:space="preserve">    padding: 0;</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    background-color: #262a2f;</t>
+          <t xml:space="preserve">    font-family: 'Poppins', sans-serif;</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="15" t="inlineStr">
         <is>
+          <t xml:space="preserve">    box-sizing: border-box;</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="15" t="inlineStr">
+        <is>
           <t>}</t>
         </is>
       </c>
     </row>
-    <row r="175">
-      <c r="A175" s="15" t="inlineStr"/>
-    </row>
     <row r="176">
-      <c r="A176" s="15" t="inlineStr">
-        <is>
-          <t>.container{</t>
-        </is>
-      </c>
+      <c r="A176" s="15" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    width : 400px;</t>
+          <t>:root {</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    background-color: white;</t>
+          <t xml:space="preserve">    --primary-color: #494eea;</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    border-radius: 10px;  </t>
+          <t xml:space="preserve">    --bg-color: #262a2f;</t>
         </is>
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="15" t="inlineStr"/>
+      <c r="A180" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    --error-color: #e88484;</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    /* Centering the div */</t>
+          <t>}</t>
         </is>
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    padding: 25px 35px;</t>
-        </is>
-      </c>
+      <c r="A182" s="15" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    position:absolute;</t>
+          <t>body{</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    top : 50%;</t>
+          <t xml:space="preserve">    background-color: var(--bg-color);</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    left: 50%;</t>
+          <t>}</t>
         </is>
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    transform: translate(-50%, -50%);  </t>
-        </is>
-      </c>
+      <c r="A186" s="15" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" s="15" t="inlineStr">
         <is>
-          <t>}</t>
+          <t>.container{</t>
         </is>
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="15" t="inlineStr"/>
+      <c r="A188" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    width: 400px;</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="15" t="inlineStr">
         <is>
-          <t>.container p{</t>
+          <t xml:space="preserve">    max-width: 90%; /* Ensure responsiveness on smaller screens */</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    font-weight: 600;</t>
+          <t xml:space="preserve">    background-color: white;</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    font-size: 15px;</t>
+          <t xml:space="preserve">    border-radius: 10px;  </t>
         </is>
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    margin-bottom: 8px;</t>
-        </is>
-      </c>
+      <c r="A192" s="15" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" s="15" t="inlineStr">
         <is>
-          <t>}</t>
+          <t xml:space="preserve">    /* Centering the div */</t>
         </is>
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="15" t="inlineStr"/>
+      <c r="A194" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    padding: 25px 35px;</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="15" t="inlineStr">
         <is>
-          <t>.container input{</t>
+          <t xml:space="preserve">    position: absolute;</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    width: 100%;</t>
+          <t xml:space="preserve">    top: 50%;</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    height: 50px;</t>
+          <t xml:space="preserve">    left: 50%;</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    border: 1px solid #494eea;</t>
+          <t xml:space="preserve">    transform: translate(-50%, -50%);  </t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    outline: 0;</t>
+          <t>}</t>
         </is>
       </c>
     </row>
     <row r="200">
-      <c r="A200" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    padding: 10px;</t>
-        </is>
-      </c>
+      <c r="A200" s="15" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    margin: 10px 0 20px;</t>
+          <t>.container p{</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    border-radius: 5px;</t>
+          <t xml:space="preserve">    font-weight: 600;</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="15" t="inlineStr">
         <is>
-          <t>}</t>
+          <t xml:space="preserve">    font-size: 15px;</t>
         </is>
       </c>
     </row>
     <row r="204">
-      <c r="A204" s="15" t="inlineStr"/>
+      <c r="A204" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    margin-bottom: 8px;</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="15" t="inlineStr">
         <is>
-          <t>.container button{</t>
+          <t>}</t>
         </is>
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    width: 100%;</t>
-        </is>
-      </c>
+      <c r="A206" s="15" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    height: 50px;</t>
+          <t>.container input{</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    border : 0;</t>
+          <t xml:space="preserve">    width: 100%;</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    background-color: #494eea;</t>
+          <t xml:space="preserve">    height: 50px;</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    color: white;</t>
+          <t xml:space="preserve">    border: 1px solid var(--primary-color);</t>
         </is>
       </c>
     </row>
@@ -2915,135 +2975,139 @@
     <row r="212">
       <c r="A212" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    border-radius: 5px;</t>
+          <t xml:space="preserve">    padding: 10px;</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    margin:20px 0;</t>
+          <t xml:space="preserve">    margin: 10px 0 20px;</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    font-weight: 500;</t>
+          <t xml:space="preserve">    border-radius: 5px;</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    cursor: pointer;</t>
+          <t>}</t>
         </is>
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    transition: background-color 0.2s;</t>
-        </is>
-      </c>
+      <c r="A216" s="15" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" s="15" t="inlineStr">
         <is>
-          <t>}</t>
+          <t>.container input:focus {</t>
         </is>
       </c>
     </row>
     <row r="218">
-      <c r="A218" s="15" t="inlineStr"/>
+      <c r="A218" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    border-width: 2px;</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="15" t="inlineStr">
         <is>
-          <t>.container button:hover {</t>
+          <t>}</t>
         </is>
       </c>
     </row>
     <row r="220">
-      <c r="A220" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    background-color: #3a3fb8;</t>
-        </is>
-      </c>
+      <c r="A220" s="15" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" s="15" t="inlineStr">
         <is>
-          <t>}</t>
+          <t>.container button{</t>
         </is>
       </c>
     </row>
     <row r="222">
-      <c r="A222" s="15" t="inlineStr"/>
+      <c r="A222" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    width: 100%;</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="15" t="inlineStr">
         <is>
-          <t>#imgBox{</t>
+          <t xml:space="preserve">    height: 50px;</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    width: 100%;</t>
+          <t xml:space="preserve">    border: 0;</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    display: flex;</t>
+          <t xml:space="preserve">    background-color: var(--primary-color);</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    justify-content: center;</t>
+          <t xml:space="preserve">    color: white;</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    min-height: 150px;</t>
+          <t xml:space="preserve">    outline: 0;</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    align-items: center;</t>
+          <t xml:space="preserve">    border-radius: 5px;</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="15" t="inlineStr">
         <is>
-          <t>}</t>
+          <t xml:space="preserve">    margin: 20px 0;</t>
         </is>
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="15" t="inlineStr"/>
+      <c r="A230" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    font-weight: 500;</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="15" t="inlineStr">
         <is>
-          <t>#Qr-Image {</t>
+          <t xml:space="preserve">    cursor: pointer;</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    display: none; /* Hidden until loaded */</t>
+          <t xml:space="preserve">    transition: background 0.3s ease;</t>
         </is>
       </c>
     </row>
@@ -3060,68 +3124,154 @@
     <row r="235">
       <c r="A235" s="15" t="inlineStr">
         <is>
-          <t>.invalid-input{</t>
+          <t>.container button:hover {</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    border: 2px solid #ff0000;</t>
+          <t xml:space="preserve">    background-color: #3b3fcc;</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    background-color: rgb(232, 132, 132);</t>
+          <t>}</t>
         </is>
       </c>
     </row>
     <row r="238">
-      <c r="A238" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    color: white;</t>
-        </is>
-      </c>
+      <c r="A238" s="15" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    border-radius: 3px;</t>
+          <t>#imgBox{</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    padding: 5px;</t>
+          <t xml:space="preserve">    width: 100%; /* Fixed missing unit */</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    text-align: center;</t>
+          <t xml:space="preserve">    display: flex;</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    width: 100%;</t>
+          <t xml:space="preserve">    justify-content: center;</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="15" t="inlineStr">
         <is>
-          <t>}</t>
+          <t xml:space="preserve">    overflow: hidden; /* Prevent overflow if image is too large */</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="15" t="inlineStr">
+        <is>
+          <t>}</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="15" t="inlineStr"/>
+    </row>
+    <row r="246">
+      <c r="A246" s="15" t="inlineStr">
+        <is>
+          <t>#imgBox img {</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    max-width: 100%;</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="15" t="inlineStr">
+        <is>
+          <t>}</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="15" t="inlineStr"/>
+    </row>
+    <row r="250">
+      <c r="A250" s="15" t="inlineStr">
+        <is>
+          <t>.invalid-input{</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    border: 2px solid red !important;</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    background-color: var(--error-color);</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    color: white;</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    border-radius: 3px;</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    padding: 5px;</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    transition: all 0.3s ease;</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="15" t="inlineStr">
+        <is>
+          <t>}</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="15" t="inlineStr">
         <is>
           <t>```</t>
         </is>

</xml_diff>